<commit_message>
Add cache-busting headers and timestamp to prevent API caching
</commit_message>
<xml_diff>
--- a/salaries.xlsx
+++ b/salaries.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\20251204\sical\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{230296CC-A30A-42B6-B45E-8580034738B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD1DEFA7-4DC8-48C8-9D6B-F5276AC58CF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1800" yWindow="170" windowWidth="17205" windowHeight="9910" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="salaries" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="14">
   <si>
     <t>id</t>
   </si>
@@ -73,6 +73,10 @@
   </si>
   <si>
     <t>欧阳七</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>欧阳八</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -627,7 +631,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E73"/>
   <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="13.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="8.7265625" style="1"/>
@@ -1675,6 +1679,210 @@
         <v>400000</v>
       </c>
     </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A62" s="1">
+        <v>61</v>
+      </c>
+      <c r="B62" s="1">
+        <v>6</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62" s="1">
+        <v>202401</v>
+      </c>
+      <c r="E62" s="1">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A63" s="1">
+        <v>62</v>
+      </c>
+      <c r="B63" s="1">
+        <v>6</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D63" s="1">
+        <v>202402</v>
+      </c>
+      <c r="E63" s="1">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A64" s="1">
+        <v>63</v>
+      </c>
+      <c r="B64" s="1">
+        <v>6</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D64" s="1">
+        <v>202403</v>
+      </c>
+      <c r="E64" s="1">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A65" s="1">
+        <v>64</v>
+      </c>
+      <c r="B65" s="1">
+        <v>6</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D65" s="1">
+        <v>202404</v>
+      </c>
+      <c r="E65" s="1">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A66" s="1">
+        <v>65</v>
+      </c>
+      <c r="B66" s="1">
+        <v>6</v>
+      </c>
+      <c r="C66" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D66" s="1">
+        <v>202405</v>
+      </c>
+      <c r="E66" s="1">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A67" s="1">
+        <v>66</v>
+      </c>
+      <c r="B67" s="1">
+        <v>6</v>
+      </c>
+      <c r="C67" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D67" s="1">
+        <v>202406</v>
+      </c>
+      <c r="E67" s="1">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A68" s="1">
+        <v>67</v>
+      </c>
+      <c r="B68" s="1">
+        <v>6</v>
+      </c>
+      <c r="C68" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D68" s="1">
+        <v>202407</v>
+      </c>
+      <c r="E68" s="1">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A69" s="1">
+        <v>68</v>
+      </c>
+      <c r="B69" s="1">
+        <v>6</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D69" s="1">
+        <v>202408</v>
+      </c>
+      <c r="E69" s="1">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A70" s="1">
+        <v>69</v>
+      </c>
+      <c r="B70" s="1">
+        <v>6</v>
+      </c>
+      <c r="C70" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D70" s="1">
+        <v>202409</v>
+      </c>
+      <c r="E70" s="1">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A71" s="1">
+        <v>70</v>
+      </c>
+      <c r="B71" s="1">
+        <v>6</v>
+      </c>
+      <c r="C71" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D71" s="1">
+        <v>202410</v>
+      </c>
+      <c r="E71" s="1">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A72" s="1">
+        <v>71</v>
+      </c>
+      <c r="B72" s="1">
+        <v>6</v>
+      </c>
+      <c r="C72" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D72" s="1">
+        <v>202411</v>
+      </c>
+      <c r="E72" s="1">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A73" s="1">
+        <v>72</v>
+      </c>
+      <c r="B73" s="1">
+        <v>6</v>
+      </c>
+      <c r="C73" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D73" s="1">
+        <v>202412</v>
+      </c>
+      <c r="E73" s="1">
+        <v>8000</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add investigation API and simplify results query to ensure all records are returned
</commit_message>
<xml_diff>
--- a/salaries.xlsx
+++ b/salaries.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\20251204\sical\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD1DEFA7-4DC8-48C8-9D6B-F5276AC58CF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA276CC8-E887-436B-AC6D-61CDAEA53211}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="16">
   <si>
     <t>id</t>
   </si>
@@ -77,6 +77,14 @@
   </si>
   <si>
     <t>欧阳八</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>欧阳九</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>欧阳时</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -631,7 +639,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E73"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="13.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="8.7265625" style="1"/>
@@ -1883,6 +1891,414 @@
         <v>8000</v>
       </c>
     </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A74" s="1">
+        <v>73</v>
+      </c>
+      <c r="B74" s="1">
+        <v>7</v>
+      </c>
+      <c r="C74" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D74" s="1">
+        <v>202401</v>
+      </c>
+      <c r="E74" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A75" s="1">
+        <v>74</v>
+      </c>
+      <c r="B75" s="1">
+        <v>7</v>
+      </c>
+      <c r="C75" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D75" s="1">
+        <v>202402</v>
+      </c>
+      <c r="E75" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A76" s="1">
+        <v>75</v>
+      </c>
+      <c r="B76" s="1">
+        <v>7</v>
+      </c>
+      <c r="C76" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D76" s="1">
+        <v>202403</v>
+      </c>
+      <c r="E76" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A77" s="1">
+        <v>76</v>
+      </c>
+      <c r="B77" s="1">
+        <v>7</v>
+      </c>
+      <c r="C77" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D77" s="1">
+        <v>202404</v>
+      </c>
+      <c r="E77" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A78" s="1">
+        <v>77</v>
+      </c>
+      <c r="B78" s="1">
+        <v>7</v>
+      </c>
+      <c r="C78" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D78" s="1">
+        <v>202405</v>
+      </c>
+      <c r="E78" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A79" s="1">
+        <v>78</v>
+      </c>
+      <c r="B79" s="1">
+        <v>7</v>
+      </c>
+      <c r="C79" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D79" s="1">
+        <v>202406</v>
+      </c>
+      <c r="E79" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A80" s="1">
+        <v>79</v>
+      </c>
+      <c r="B80" s="1">
+        <v>7</v>
+      </c>
+      <c r="C80" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D80" s="1">
+        <v>202407</v>
+      </c>
+      <c r="E80" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A81" s="1">
+        <v>80</v>
+      </c>
+      <c r="B81" s="1">
+        <v>7</v>
+      </c>
+      <c r="C81" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D81" s="1">
+        <v>202408</v>
+      </c>
+      <c r="E81" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A82" s="1">
+        <v>81</v>
+      </c>
+      <c r="B82" s="1">
+        <v>7</v>
+      </c>
+      <c r="C82" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D82" s="1">
+        <v>202409</v>
+      </c>
+      <c r="E82" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A83" s="1">
+        <v>82</v>
+      </c>
+      <c r="B83" s="1">
+        <v>7</v>
+      </c>
+      <c r="C83" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D83" s="1">
+        <v>202410</v>
+      </c>
+      <c r="E83" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A84" s="1">
+        <v>83</v>
+      </c>
+      <c r="B84" s="1">
+        <v>7</v>
+      </c>
+      <c r="C84" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D84" s="1">
+        <v>202411</v>
+      </c>
+      <c r="E84" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A85" s="1">
+        <v>84</v>
+      </c>
+      <c r="B85" s="1">
+        <v>7</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D85" s="1">
+        <v>202412</v>
+      </c>
+      <c r="E85" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A86" s="1">
+        <v>73</v>
+      </c>
+      <c r="B86" s="1">
+        <v>8</v>
+      </c>
+      <c r="C86" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D86" s="1">
+        <v>202401</v>
+      </c>
+      <c r="E86" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A87" s="1">
+        <v>74</v>
+      </c>
+      <c r="B87" s="1">
+        <v>8</v>
+      </c>
+      <c r="C87" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D87" s="1">
+        <v>202402</v>
+      </c>
+      <c r="E87" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A88" s="1">
+        <v>75</v>
+      </c>
+      <c r="B88" s="1">
+        <v>8</v>
+      </c>
+      <c r="C88" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D88" s="1">
+        <v>202403</v>
+      </c>
+      <c r="E88" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A89" s="1">
+        <v>76</v>
+      </c>
+      <c r="B89" s="1">
+        <v>8</v>
+      </c>
+      <c r="C89" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D89" s="1">
+        <v>202404</v>
+      </c>
+      <c r="E89" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A90" s="1">
+        <v>77</v>
+      </c>
+      <c r="B90" s="1">
+        <v>8</v>
+      </c>
+      <c r="C90" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D90" s="1">
+        <v>202405</v>
+      </c>
+      <c r="E90" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A91" s="1">
+        <v>78</v>
+      </c>
+      <c r="B91" s="1">
+        <v>8</v>
+      </c>
+      <c r="C91" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D91" s="1">
+        <v>202406</v>
+      </c>
+      <c r="E91" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A92" s="1">
+        <v>79</v>
+      </c>
+      <c r="B92" s="1">
+        <v>8</v>
+      </c>
+      <c r="C92" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D92" s="1">
+        <v>202407</v>
+      </c>
+      <c r="E92" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A93" s="1">
+        <v>80</v>
+      </c>
+      <c r="B93" s="1">
+        <v>8</v>
+      </c>
+      <c r="C93" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D93" s="1">
+        <v>202408</v>
+      </c>
+      <c r="E93" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A94" s="1">
+        <v>81</v>
+      </c>
+      <c r="B94" s="1">
+        <v>8</v>
+      </c>
+      <c r="C94" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D94" s="1">
+        <v>202409</v>
+      </c>
+      <c r="E94" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A95" s="1">
+        <v>82</v>
+      </c>
+      <c r="B95" s="1">
+        <v>8</v>
+      </c>
+      <c r="C95" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D95" s="1">
+        <v>202410</v>
+      </c>
+      <c r="E95" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A96" s="1">
+        <v>83</v>
+      </c>
+      <c r="B96" s="1">
+        <v>8</v>
+      </c>
+      <c r="C96" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D96" s="1">
+        <v>202411</v>
+      </c>
+      <c r="E96" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A97" s="1">
+        <v>84</v>
+      </c>
+      <c r="B97" s="1">
+        <v>8</v>
+      </c>
+      <c r="C97" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D97" s="1">
+        <v>202412</v>
+      </c>
+      <c r="E97" s="1">
+        <v>9000</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add more debug info to results API to track actual record count
</commit_message>
<xml_diff>
--- a/salaries.xlsx
+++ b/salaries.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\20251204\sical\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA276CC8-E887-436B-AC6D-61CDAEA53211}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F0F9281-390E-4098-AB27-BA503B1872FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="17">
   <si>
     <t>id</t>
   </si>
@@ -85,6 +85,10 @@
   </si>
   <si>
     <t>欧阳时</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>欧阳时以</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -639,7 +643,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E97"/>
+  <dimension ref="A1:E109"/>
   <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="13.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="8.7265625" style="1"/>
@@ -2299,6 +2303,210 @@
         <v>9000</v>
       </c>
     </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A98" s="1">
+        <v>85</v>
+      </c>
+      <c r="B98" s="1">
+        <v>9</v>
+      </c>
+      <c r="C98" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D98" s="1">
+        <v>202401</v>
+      </c>
+      <c r="E98" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A99" s="1">
+        <v>86</v>
+      </c>
+      <c r="B99" s="1">
+        <v>9</v>
+      </c>
+      <c r="C99" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D99" s="1">
+        <v>202402</v>
+      </c>
+      <c r="E99" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A100" s="1">
+        <v>87</v>
+      </c>
+      <c r="B100" s="1">
+        <v>9</v>
+      </c>
+      <c r="C100" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D100" s="1">
+        <v>202403</v>
+      </c>
+      <c r="E100" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A101" s="1">
+        <v>88</v>
+      </c>
+      <c r="B101" s="1">
+        <v>9</v>
+      </c>
+      <c r="C101" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D101" s="1">
+        <v>202404</v>
+      </c>
+      <c r="E101" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A102" s="1">
+        <v>89</v>
+      </c>
+      <c r="B102" s="1">
+        <v>9</v>
+      </c>
+      <c r="C102" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D102" s="1">
+        <v>202405</v>
+      </c>
+      <c r="E102" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A103" s="1">
+        <v>90</v>
+      </c>
+      <c r="B103" s="1">
+        <v>9</v>
+      </c>
+      <c r="C103" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D103" s="1">
+        <v>202406</v>
+      </c>
+      <c r="E103" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A104" s="1">
+        <v>91</v>
+      </c>
+      <c r="B104" s="1">
+        <v>9</v>
+      </c>
+      <c r="C104" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D104" s="1">
+        <v>202407</v>
+      </c>
+      <c r="E104" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A105" s="1">
+        <v>92</v>
+      </c>
+      <c r="B105" s="1">
+        <v>9</v>
+      </c>
+      <c r="C105" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D105" s="1">
+        <v>202408</v>
+      </c>
+      <c r="E105" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A106" s="1">
+        <v>93</v>
+      </c>
+      <c r="B106" s="1">
+        <v>9</v>
+      </c>
+      <c r="C106" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D106" s="1">
+        <v>202409</v>
+      </c>
+      <c r="E106" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A107" s="1">
+        <v>94</v>
+      </c>
+      <c r="B107" s="1">
+        <v>9</v>
+      </c>
+      <c r="C107" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D107" s="1">
+        <v>202410</v>
+      </c>
+      <c r="E107" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A108" s="1">
+        <v>95</v>
+      </c>
+      <c r="B108" s="1">
+        <v>9</v>
+      </c>
+      <c r="C108" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D108" s="1">
+        <v>202411</v>
+      </c>
+      <c r="E108" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A109" s="1">
+        <v>96</v>
+      </c>
+      <c r="B109" s="1">
+        <v>9</v>
+      </c>
+      <c r="C109" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D109" s="1">
+        <v>202412</v>
+      </c>
+      <c r="E109" s="1">
+        <v>9000</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add fresh API endpoint to bypass Supabase cache and ensure real-time data
</commit_message>
<xml_diff>
--- a/salaries.xlsx
+++ b/salaries.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\20251204\sical\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F0F9281-390E-4098-AB27-BA503B1872FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2004D1D8-F4C4-46BB-95B4-2D9071286E2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="18">
   <si>
     <t>id</t>
   </si>
@@ -89,6 +89,10 @@
   </si>
   <si>
     <t>欧阳时以</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>欧阳时尔</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -643,7 +647,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E109"/>
+  <dimension ref="A1:E121"/>
   <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="13.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="8.7265625" style="1"/>
@@ -2507,6 +2511,210 @@
         <v>9000</v>
       </c>
     </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A110" s="1">
+        <v>97</v>
+      </c>
+      <c r="B110" s="1">
+        <v>10</v>
+      </c>
+      <c r="C110" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D110" s="1">
+        <v>202401</v>
+      </c>
+      <c r="E110" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A111" s="1">
+        <v>98</v>
+      </c>
+      <c r="B111" s="1">
+        <v>10</v>
+      </c>
+      <c r="C111" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D111" s="1">
+        <v>202402</v>
+      </c>
+      <c r="E111" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A112" s="1">
+        <v>99</v>
+      </c>
+      <c r="B112" s="1">
+        <v>10</v>
+      </c>
+      <c r="C112" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D112" s="1">
+        <v>202403</v>
+      </c>
+      <c r="E112" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A113" s="1">
+        <v>100</v>
+      </c>
+      <c r="B113" s="1">
+        <v>10</v>
+      </c>
+      <c r="C113" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D113" s="1">
+        <v>202404</v>
+      </c>
+      <c r="E113" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A114" s="1">
+        <v>101</v>
+      </c>
+      <c r="B114" s="1">
+        <v>10</v>
+      </c>
+      <c r="C114" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D114" s="1">
+        <v>202405</v>
+      </c>
+      <c r="E114" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A115" s="1">
+        <v>102</v>
+      </c>
+      <c r="B115" s="1">
+        <v>10</v>
+      </c>
+      <c r="C115" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D115" s="1">
+        <v>202406</v>
+      </c>
+      <c r="E115" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A116" s="1">
+        <v>103</v>
+      </c>
+      <c r="B116" s="1">
+        <v>10</v>
+      </c>
+      <c r="C116" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D116" s="1">
+        <v>202407</v>
+      </c>
+      <c r="E116" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A117" s="1">
+        <v>104</v>
+      </c>
+      <c r="B117" s="1">
+        <v>10</v>
+      </c>
+      <c r="C117" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D117" s="1">
+        <v>202408</v>
+      </c>
+      <c r="E117" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A118" s="1">
+        <v>105</v>
+      </c>
+      <c r="B118" s="1">
+        <v>10</v>
+      </c>
+      <c r="C118" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D118" s="1">
+        <v>202409</v>
+      </c>
+      <c r="E118" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A119" s="1">
+        <v>106</v>
+      </c>
+      <c r="B119" s="1">
+        <v>10</v>
+      </c>
+      <c r="C119" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D119" s="1">
+        <v>202410</v>
+      </c>
+      <c r="E119" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A120" s="1">
+        <v>107</v>
+      </c>
+      <c r="B120" s="1">
+        <v>10</v>
+      </c>
+      <c r="C120" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D120" s="1">
+        <v>202411</v>
+      </c>
+      <c r="E120" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A121" s="1">
+        <v>108</v>
+      </c>
+      <c r="B121" s="1">
+        <v>10</v>
+      </c>
+      <c r="C121" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D121" s="1">
+        <v>202412</v>
+      </c>
+      <c r="E121" s="1">
+        <v>9000</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Implement aggressive cache-busting solution for real-time data updates
- Add results-raw API with fresh Supabase client per request
- Create database functions for direct SQL queries
- Implement multi-step refresh strategy in frontend
- Add detailed logging for debugging cache issues
- Create database setup API for manual function creation

This should completely resolve Supabase caching issues preventing real-time updates

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/salaries.xlsx
+++ b/salaries.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\20251204\sical\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2004D1D8-F4C4-46BB-95B4-2D9071286E2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADC16DCD-F8ED-4893-B322-46344C5242BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="19">
   <si>
     <t>id</t>
   </si>
@@ -93,6 +93,10 @@
   </si>
   <si>
     <t>欧阳时尔</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>欧阳时森</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -647,7 +651,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E121"/>
+  <dimension ref="A1:E133"/>
   <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="13.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="8.7265625" style="1"/>
@@ -2715,6 +2719,210 @@
         <v>9000</v>
       </c>
     </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A122" s="1">
+        <v>109</v>
+      </c>
+      <c r="B122" s="1">
+        <v>11</v>
+      </c>
+      <c r="C122" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D122" s="1">
+        <v>202401</v>
+      </c>
+      <c r="E122" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A123" s="1">
+        <v>110</v>
+      </c>
+      <c r="B123" s="1">
+        <v>11</v>
+      </c>
+      <c r="C123" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D123" s="1">
+        <v>202402</v>
+      </c>
+      <c r="E123" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A124" s="1">
+        <v>111</v>
+      </c>
+      <c r="B124" s="1">
+        <v>11</v>
+      </c>
+      <c r="C124" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D124" s="1">
+        <v>202403</v>
+      </c>
+      <c r="E124" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A125" s="1">
+        <v>112</v>
+      </c>
+      <c r="B125" s="1">
+        <v>11</v>
+      </c>
+      <c r="C125" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D125" s="1">
+        <v>202404</v>
+      </c>
+      <c r="E125" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A126" s="1">
+        <v>113</v>
+      </c>
+      <c r="B126" s="1">
+        <v>11</v>
+      </c>
+      <c r="C126" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D126" s="1">
+        <v>202405</v>
+      </c>
+      <c r="E126" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A127" s="1">
+        <v>114</v>
+      </c>
+      <c r="B127" s="1">
+        <v>11</v>
+      </c>
+      <c r="C127" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D127" s="1">
+        <v>202406</v>
+      </c>
+      <c r="E127" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A128" s="1">
+        <v>115</v>
+      </c>
+      <c r="B128" s="1">
+        <v>11</v>
+      </c>
+      <c r="C128" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D128" s="1">
+        <v>202407</v>
+      </c>
+      <c r="E128" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A129" s="1">
+        <v>116</v>
+      </c>
+      <c r="B129" s="1">
+        <v>11</v>
+      </c>
+      <c r="C129" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D129" s="1">
+        <v>202408</v>
+      </c>
+      <c r="E129" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A130" s="1">
+        <v>117</v>
+      </c>
+      <c r="B130" s="1">
+        <v>11</v>
+      </c>
+      <c r="C130" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D130" s="1">
+        <v>202409</v>
+      </c>
+      <c r="E130" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A131" s="1">
+        <v>118</v>
+      </c>
+      <c r="B131" s="1">
+        <v>11</v>
+      </c>
+      <c r="C131" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D131" s="1">
+        <v>202410</v>
+      </c>
+      <c r="E131" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A132" s="1">
+        <v>119</v>
+      </c>
+      <c r="B132" s="1">
+        <v>11</v>
+      </c>
+      <c r="C132" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D132" s="1">
+        <v>202411</v>
+      </c>
+      <c r="E132" s="1">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A133" s="1">
+        <v>120</v>
+      </c>
+      <c r="B133" s="1">
+        <v>11</v>
+      </c>
+      <c r="C133" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D133" s="1">
+        <v>202412</v>
+      </c>
+      <c r="E133" s="1">
+        <v>9000</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix multi-city support and improve data validation
- Add city field to salary data and calculation results
- Fix employee grouping to use employee_id instead of name
- Handle duplicate records by taking the latest entry
- Add financial rounding to 2 decimal places
- Add Excel data validation with detailed error messages
- Match employee city with city standards for calculations
- Update results page to display employee_id and city
- Remove debug/test API endpoints

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/salaries.xlsx
+++ b/salaries.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\20251204\sical\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADC16DCD-F8ED-4893-B322-46344C5242BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4863E6E-ADF9-48E4-9D83-DAF679A91850}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10276" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="salaries" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="21">
   <si>
     <t>id</t>
   </si>
@@ -99,6 +99,14 @@
     <t>欧阳时森</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
+  <si>
+    <t>city</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>佛山</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -155,7 +163,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -169,6 +177,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -651,18 +665,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E133"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="13.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:F133"/>
+  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.7265625" style="1"/>
-    <col min="2" max="2" width="19.08984375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="26.08984375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="14.7265625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="23.54296875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="26.08984375" customWidth="1"/>
+    <col min="1" max="1" width="8.73046875" style="1"/>
+    <col min="2" max="2" width="19.06640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="26.06640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="14.73046875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="23.53125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="26.06640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -678,8 +692,11 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F1" s="6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -695,8 +712,11 @@
       <c r="E2" s="1">
         <v>30000</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F2" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -712,8 +732,11 @@
       <c r="E3" s="1">
         <v>29000</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F3" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -729,8 +752,11 @@
       <c r="E4" s="1">
         <v>31000</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F4" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -746,8 +772,11 @@
       <c r="E5" s="1">
         <v>30000</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F5" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -763,8 +792,11 @@
       <c r="E6" s="1">
         <v>29000</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F6" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -780,8 +812,11 @@
       <c r="E7" s="1">
         <v>31000</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F7" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -797,8 +832,11 @@
       <c r="E8" s="1">
         <v>30000</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F8" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -814,8 +852,11 @@
       <c r="E9" s="1">
         <v>29000</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F9" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -831,8 +872,11 @@
       <c r="E10" s="1">
         <v>31000</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F10" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -848,8 +892,11 @@
       <c r="E11" s="1">
         <v>30000</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F11" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -865,8 +912,11 @@
       <c r="E12" s="1">
         <v>29000</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F12" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -882,8 +932,11 @@
       <c r="E13" s="1">
         <v>31000</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F13" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -899,8 +952,11 @@
       <c r="E14" s="1">
         <v>15000</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F14" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -916,8 +972,11 @@
       <c r="E15" s="1">
         <v>14000</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F15" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -933,8 +992,11 @@
       <c r="E16" s="1">
         <v>16000</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F16" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -950,8 +1012,11 @@
       <c r="E17" s="1">
         <v>15000</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F17" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -967,8 +1032,11 @@
       <c r="E18" s="1">
         <v>14000</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F18" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -984,8 +1052,11 @@
       <c r="E19" s="1">
         <v>16000</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F19" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -1001,8 +1072,11 @@
       <c r="E20" s="1">
         <v>15000</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F20" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>20</v>
       </c>
@@ -1018,8 +1092,11 @@
       <c r="E21" s="1">
         <v>14000</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F21" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>21</v>
       </c>
@@ -1035,8 +1112,11 @@
       <c r="E22" s="1">
         <v>16000</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F22" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>22</v>
       </c>
@@ -1052,8 +1132,11 @@
       <c r="E23" s="1">
         <v>15000</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F23" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>23</v>
       </c>
@@ -1069,8 +1152,11 @@
       <c r="E24" s="1">
         <v>14000</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F24" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>24</v>
       </c>
@@ -1086,8 +1172,11 @@
       <c r="E25" s="1">
         <v>16000</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F25" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>25</v>
       </c>
@@ -1103,8 +1192,11 @@
       <c r="E26" s="1">
         <v>4000</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F26" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>26</v>
       </c>
@@ -1120,8 +1212,11 @@
       <c r="E27" s="1">
         <v>3900</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F27" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>27</v>
       </c>
@@ -1137,8 +1232,11 @@
       <c r="E28" s="1">
         <v>4100</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F28" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>28</v>
       </c>
@@ -1154,8 +1252,11 @@
       <c r="E29" s="1">
         <v>4000</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F29" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>29</v>
       </c>
@@ -1171,8 +1272,11 @@
       <c r="E30" s="1">
         <v>3900</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F30" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>30</v>
       </c>
@@ -1188,8 +1292,11 @@
       <c r="E31" s="1">
         <v>4100</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F31" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>31</v>
       </c>
@@ -1205,8 +1312,11 @@
       <c r="E32" s="1">
         <v>4000</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F32" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
         <v>32</v>
       </c>
@@ -1222,8 +1332,11 @@
       <c r="E33" s="1">
         <v>3900</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F33" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="1">
         <v>33</v>
       </c>
@@ -1239,8 +1352,11 @@
       <c r="E34" s="1">
         <v>4100</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F34" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="1">
         <v>34</v>
       </c>
@@ -1256,8 +1372,11 @@
       <c r="E35" s="1">
         <v>4000</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F35" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="1">
         <v>35</v>
       </c>
@@ -1273,8 +1392,11 @@
       <c r="E36" s="1">
         <v>3900</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F36" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="1">
         <v>36</v>
       </c>
@@ -1290,8 +1412,11 @@
       <c r="E37" s="1">
         <v>4100</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F37" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="1">
         <v>37</v>
       </c>
@@ -1307,8 +1432,11 @@
       <c r="E38" s="1">
         <v>4000</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F38" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="1">
         <v>38</v>
       </c>
@@ -1324,8 +1452,11 @@
       <c r="E39" s="1">
         <v>3900</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F39" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="1">
         <v>39</v>
       </c>
@@ -1341,8 +1472,11 @@
       <c r="E40" s="1">
         <v>4100</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F40" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="1">
         <v>40</v>
       </c>
@@ -1358,8 +1492,11 @@
       <c r="E41" s="1">
         <v>4000</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F41" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" s="1">
         <v>41</v>
       </c>
@@ -1375,8 +1512,11 @@
       <c r="E42" s="1">
         <v>3900</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F42" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" s="1">
         <v>42</v>
       </c>
@@ -1392,8 +1532,11 @@
       <c r="E43" s="1">
         <v>4100</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F43" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" s="1">
         <v>43</v>
       </c>
@@ -1409,8 +1552,11 @@
       <c r="E44" s="1">
         <v>4000</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F44" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" s="1">
         <v>44</v>
       </c>
@@ -1426,8 +1572,11 @@
       <c r="E45" s="1">
         <v>3900</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F45" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" s="1">
         <v>45</v>
       </c>
@@ -1443,8 +1592,11 @@
       <c r="E46" s="1">
         <v>4100</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F46" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" s="1">
         <v>46</v>
       </c>
@@ -1460,8 +1612,11 @@
       <c r="E47" s="1">
         <v>4000</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F47" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" s="1">
         <v>47</v>
       </c>
@@ -1477,8 +1632,11 @@
       <c r="E48" s="1">
         <v>3900</v>
       </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F48" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" s="1">
         <v>48</v>
       </c>
@@ -1494,8 +1652,11 @@
       <c r="E49" s="1">
         <v>4100</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F49" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="1">
         <v>49</v>
       </c>
@@ -1511,8 +1672,11 @@
       <c r="E50" s="1">
         <v>400000</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F50" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" s="1">
         <v>50</v>
       </c>
@@ -1528,8 +1692,11 @@
       <c r="E51" s="1">
         <v>400000</v>
       </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F51" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" s="1">
         <v>51</v>
       </c>
@@ -1545,8 +1712,11 @@
       <c r="E52" s="1">
         <v>400000</v>
       </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F52" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" s="1">
         <v>52</v>
       </c>
@@ -1562,8 +1732,11 @@
       <c r="E53" s="1">
         <v>400000</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F53" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" s="1">
         <v>53</v>
       </c>
@@ -1579,8 +1752,11 @@
       <c r="E54" s="1">
         <v>400000</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F54" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" s="1">
         <v>54</v>
       </c>
@@ -1596,8 +1772,11 @@
       <c r="E55" s="1">
         <v>400000</v>
       </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F55" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" s="1">
         <v>55</v>
       </c>
@@ -1613,8 +1792,11 @@
       <c r="E56" s="1">
         <v>400000</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F56" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" s="1">
         <v>56</v>
       </c>
@@ -1630,8 +1812,11 @@
       <c r="E57" s="1">
         <v>400000</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F57" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" s="1">
         <v>57</v>
       </c>
@@ -1647,8 +1832,11 @@
       <c r="E58" s="1">
         <v>400000</v>
       </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F58" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" s="1">
         <v>58</v>
       </c>
@@ -1664,8 +1852,11 @@
       <c r="E59" s="1">
         <v>400000</v>
       </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F59" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" s="1">
         <v>59</v>
       </c>
@@ -1681,8 +1872,11 @@
       <c r="E60" s="1">
         <v>400000</v>
       </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F60" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" s="1">
         <v>60</v>
       </c>
@@ -1698,8 +1892,11 @@
       <c r="E61" s="1">
         <v>400000</v>
       </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F61" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" s="1">
         <v>61</v>
       </c>
@@ -1715,8 +1912,11 @@
       <c r="E62" s="1">
         <v>8000</v>
       </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F62" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" s="1">
         <v>62</v>
       </c>
@@ -1732,8 +1932,11 @@
       <c r="E63" s="1">
         <v>8000</v>
       </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F63" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" s="1">
         <v>63</v>
       </c>
@@ -1749,8 +1952,11 @@
       <c r="E64" s="1">
         <v>8000</v>
       </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F64" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" s="1">
         <v>64</v>
       </c>
@@ -1766,8 +1972,11 @@
       <c r="E65" s="1">
         <v>8000</v>
       </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F65" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" s="1">
         <v>65</v>
       </c>
@@ -1783,8 +1992,11 @@
       <c r="E66" s="1">
         <v>8000</v>
       </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F66" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67" s="1">
         <v>66</v>
       </c>
@@ -1800,8 +2012,11 @@
       <c r="E67" s="1">
         <v>8000</v>
       </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F67" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" s="1">
         <v>67</v>
       </c>
@@ -1817,8 +2032,11 @@
       <c r="E68" s="1">
         <v>8000</v>
       </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F68" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69" s="1">
         <v>68</v>
       </c>
@@ -1834,8 +2052,11 @@
       <c r="E69" s="1">
         <v>8000</v>
       </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F69" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70" s="1">
         <v>69</v>
       </c>
@@ -1851,8 +2072,11 @@
       <c r="E70" s="1">
         <v>8000</v>
       </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F70" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71" s="1">
         <v>70</v>
       </c>
@@ -1868,8 +2092,11 @@
       <c r="E71" s="1">
         <v>8000</v>
       </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F71" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72" s="1">
         <v>71</v>
       </c>
@@ -1885,8 +2112,11 @@
       <c r="E72" s="1">
         <v>8000</v>
       </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F72" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73" s="1">
         <v>72</v>
       </c>
@@ -1902,8 +2132,11 @@
       <c r="E73" s="1">
         <v>8000</v>
       </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F73" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74" s="1">
         <v>73</v>
       </c>
@@ -1919,8 +2152,11 @@
       <c r="E74" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F74" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A75" s="1">
         <v>74</v>
       </c>
@@ -1936,8 +2172,11 @@
       <c r="E75" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F75" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76" s="1">
         <v>75</v>
       </c>
@@ -1953,8 +2192,11 @@
       <c r="E76" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F76" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77" s="1">
         <v>76</v>
       </c>
@@ -1970,8 +2212,11 @@
       <c r="E77" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F77" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A78" s="1">
         <v>77</v>
       </c>
@@ -1987,8 +2232,11 @@
       <c r="E78" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F78" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79" s="1">
         <v>78</v>
       </c>
@@ -2004,8 +2252,11 @@
       <c r="E79" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F79" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80" s="1">
         <v>79</v>
       </c>
@@ -2021,8 +2272,11 @@
       <c r="E80" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F80" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81" s="1">
         <v>80</v>
       </c>
@@ -2038,8 +2292,11 @@
       <c r="E81" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F81" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82" s="1">
         <v>81</v>
       </c>
@@ -2055,8 +2312,11 @@
       <c r="E82" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F82" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83" s="1">
         <v>82</v>
       </c>
@@ -2072,8 +2332,11 @@
       <c r="E83" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F83" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84" s="1">
         <v>83</v>
       </c>
@@ -2089,8 +2352,11 @@
       <c r="E84" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F84" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A85" s="1">
         <v>84</v>
       </c>
@@ -2106,8 +2372,11 @@
       <c r="E85" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F85" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A86" s="1">
         <v>73</v>
       </c>
@@ -2123,8 +2392,11 @@
       <c r="E86" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F86" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A87" s="1">
         <v>74</v>
       </c>
@@ -2140,8 +2412,11 @@
       <c r="E87" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F87" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A88" s="1">
         <v>75</v>
       </c>
@@ -2157,8 +2432,11 @@
       <c r="E88" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F88" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A89" s="1">
         <v>76</v>
       </c>
@@ -2174,8 +2452,11 @@
       <c r="E89" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F89" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A90" s="1">
         <v>77</v>
       </c>
@@ -2191,8 +2472,11 @@
       <c r="E90" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F90" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A91" s="1">
         <v>78</v>
       </c>
@@ -2208,8 +2492,11 @@
       <c r="E91" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F91" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A92" s="1">
         <v>79</v>
       </c>
@@ -2225,8 +2512,11 @@
       <c r="E92" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F92" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93" s="1">
         <v>80</v>
       </c>
@@ -2242,8 +2532,11 @@
       <c r="E93" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F93" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A94" s="1">
         <v>81</v>
       </c>
@@ -2259,8 +2552,11 @@
       <c r="E94" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F94" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A95" s="1">
         <v>82</v>
       </c>
@@ -2276,8 +2572,11 @@
       <c r="E95" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F95" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A96" s="1">
         <v>83</v>
       </c>
@@ -2293,8 +2592,11 @@
       <c r="E96" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F96" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97" s="1">
         <v>84</v>
       </c>
@@ -2310,8 +2612,11 @@
       <c r="E97" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F97" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A98" s="1">
         <v>85</v>
       </c>
@@ -2327,8 +2632,11 @@
       <c r="E98" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F98" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A99" s="1">
         <v>86</v>
       </c>
@@ -2344,8 +2652,11 @@
       <c r="E99" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F99" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A100" s="1">
         <v>87</v>
       </c>
@@ -2361,8 +2672,11 @@
       <c r="E100" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F100" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A101" s="1">
         <v>88</v>
       </c>
@@ -2378,8 +2692,11 @@
       <c r="E101" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F101" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A102" s="1">
         <v>89</v>
       </c>
@@ -2395,8 +2712,11 @@
       <c r="E102" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F102" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A103" s="1">
         <v>90</v>
       </c>
@@ -2412,8 +2732,11 @@
       <c r="E103" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F103" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A104" s="1">
         <v>91</v>
       </c>
@@ -2429,8 +2752,11 @@
       <c r="E104" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F104" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A105" s="1">
         <v>92</v>
       </c>
@@ -2446,8 +2772,11 @@
       <c r="E105" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F105" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A106" s="1">
         <v>93</v>
       </c>
@@ -2463,8 +2792,11 @@
       <c r="E106" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F106" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A107" s="1">
         <v>94</v>
       </c>
@@ -2480,8 +2812,11 @@
       <c r="E107" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F107" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A108" s="1">
         <v>95</v>
       </c>
@@ -2497,8 +2832,11 @@
       <c r="E108" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F108" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A109" s="1">
         <v>96</v>
       </c>
@@ -2514,8 +2852,11 @@
       <c r="E109" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F109" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A110" s="1">
         <v>97</v>
       </c>
@@ -2531,8 +2872,11 @@
       <c r="E110" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F110" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A111" s="1">
         <v>98</v>
       </c>
@@ -2548,8 +2892,11 @@
       <c r="E111" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F111" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A112" s="1">
         <v>99</v>
       </c>
@@ -2565,8 +2912,11 @@
       <c r="E112" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F112" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A113" s="1">
         <v>100</v>
       </c>
@@ -2582,8 +2932,11 @@
       <c r="E113" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F113" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A114" s="1">
         <v>101</v>
       </c>
@@ -2599,8 +2952,11 @@
       <c r="E114" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F114" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A115" s="1">
         <v>102</v>
       </c>
@@ -2616,8 +2972,11 @@
       <c r="E115" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F115" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A116" s="1">
         <v>103</v>
       </c>
@@ -2633,8 +2992,11 @@
       <c r="E116" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F116" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A117" s="1">
         <v>104</v>
       </c>
@@ -2650,8 +3012,11 @@
       <c r="E117" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F117" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A118" s="1">
         <v>105</v>
       </c>
@@ -2667,8 +3032,11 @@
       <c r="E118" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F118" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A119" s="1">
         <v>106</v>
       </c>
@@ -2684,8 +3052,11 @@
       <c r="E119" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F119" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A120" s="1">
         <v>107</v>
       </c>
@@ -2701,8 +3072,11 @@
       <c r="E120" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F120" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A121" s="1">
         <v>108</v>
       </c>
@@ -2718,8 +3092,11 @@
       <c r="E121" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F121" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A122" s="1">
         <v>109</v>
       </c>
@@ -2735,8 +3112,11 @@
       <c r="E122" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F122" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A123" s="1">
         <v>110</v>
       </c>
@@ -2752,8 +3132,11 @@
       <c r="E123" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F123" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A124" s="1">
         <v>111</v>
       </c>
@@ -2769,8 +3152,11 @@
       <c r="E124" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F124" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A125" s="1">
         <v>112</v>
       </c>
@@ -2786,8 +3172,11 @@
       <c r="E125" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F125" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A126" s="1">
         <v>113</v>
       </c>
@@ -2803,8 +3192,11 @@
       <c r="E126" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F126" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A127" s="1">
         <v>114</v>
       </c>
@@ -2820,8 +3212,11 @@
       <c r="E127" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F127" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A128" s="1">
         <v>115</v>
       </c>
@@ -2837,8 +3232,11 @@
       <c r="E128" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F128" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A129" s="1">
         <v>116</v>
       </c>
@@ -2854,8 +3252,11 @@
       <c r="E129" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F129" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A130" s="1">
         <v>117</v>
       </c>
@@ -2871,8 +3272,11 @@
       <c r="E130" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F130" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A131" s="1">
         <v>118</v>
       </c>
@@ -2888,8 +3292,11 @@
       <c r="E131" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F131" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A132" s="1">
         <v>119</v>
       </c>
@@ -2905,8 +3312,11 @@
       <c r="E132" s="1">
         <v>9000</v>
       </c>
-    </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F132" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A133" s="1">
         <v>120</v>
       </c>
@@ -2921,6 +3331,9 @@
       </c>
       <c r="E133" s="1">
         <v>9000</v>
+      </c>
+      <c r="F133" s="5" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>